<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-05 La carte d'Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-05.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La bulle d'Aniss</t>
+          <t>La carte d'Aniss</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour, linge, bol de savon</t>
+          <t>classe</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aniss, Raphaël, papa, maman</t>
+          <t>Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut une bulle qui va jusqu'à la chemise bleue. Il reste près du mur. Il observe d'abord. La bulle part, puis se pose.</t>
+          <t>Une barre de soleil rampe sur le plancher. Sur le bois de la chaise, un éclat de bois brille. Aniss veut la carte de l'oiseau, maintenant. Il plonge trop vite : les cartes glissent, le bruit monte. Il a besoin de calme. Papa dit les deux mots trop vite. Aniss n'entend pas. Papa les dit plus lent. Aniss refuse de foncer, observe, pioche, montre. Merci vécu. Il envoie la carte sous la chaise. Il retrouve l'éclat, reprend sans brusquer. Sur le bois, l'éclat tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le linge claque sur la corde. Une goutte tombe d'une chemise bleue. Le savon sent la fleur, dans le bol. Un cercle irisé tremble au bord. La cour est encore chaude. Tu as vu la chemise, Aniss ? Elle est bleue. Une goutte tombe. Oui. Le linge sèche. Je veux une bulle. Jusqu'à la chemise. On souffle tout doux, alors. Une pince à linge brille au soleil. Tu as vu la pince ? Elle est jaune. Oui. Elle tient la manche. En ce moment, Aniss rentre de l'école. La classe était un peu bruyante. Il reste près du mur. Le mur est chaud sous sa main. Raphaël tient déjà l'anneau. L'anneau goutte un peu de savon. J'attends un peu. Tu as besoin de calme. On peut dire comment on souffle. Le cercle irisé tremble encore. La chemise bleue attend sur la corde.</t>
+          <t>Une barre de soleil rampe sur le plancher. Dans la barre, un peu de poussière flotte. Les crayons sentent le bois, près du mur. Une chaise racle, puis s'arrête. Le carton de cartes attend sous la lumière. Dedans, les cartes glissent un peu. Sur le bois de la chaise, un éclat de bois brille. Il est petit, papa. C'est le bois, sous le soleil. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le cartable attend près de la porte. La fermeture du cartable est un peu froide. Je veux la carte de l'oiseau, maintenant ! Avant de partir ? Oui, tout de suite ! En ce moment, Aniss plonge la main dans le carton. Les cartes glissent contre ses doigts. Une carte tombe, puis une autre. La chaise racle plus fort. Papa parle à maman, près de la porte. Le cartable est près du banc. Oui, avec la fermeture. Papa, l'oiseau ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? La carte va partir. Aniss plonge trop vite, une deuxième fois. Le carton penche, puis se recale. L'oiseau disparaît sous les autres cartes. Oh. L'éclat de bois tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça fait trop de bruit, maman. Ses épaules tombent un peu. Il recule jusqu'au mur. Ses mains touchent le mur, plates. Aniss a besoin de calme. Papa se baisse à sa hauteur. Tu regardes le carton ? Oui, papa. Les crayons sentent le bois, ici. On pioche. On montre. Les deux mots passent trop vite, dans le bruit. Je n'ai pas entendu. Aniss serre le mur contre ses paumes. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le linge claque sur la corde. Une goutte tombe d'une chemise bleue. Le savon sent la fleur, dans le bol. Un cercle irisé tremble au bord. La cour est encore chaude. Tu as vu la chemise, Aniss ? Elle est bleue. Une goutte tombe. Oui. Le linge sèche. Je veux une bulle. Jusqu'à la chemise. On souffle tout doux, alors. Une pince à linge brille au soleil. Tu as vu la pince ? Elle est jaune. Oui. Elle tient la manche. En ce moment, Aniss rentre de l'école. La classe était un peu bruyante. Il reste près du mur. Le mur est chaud sous sa main. Raphaël tient déjà l'anneau. L'anneau goutte un peu de savon. J'attends un peu. Tu as besoin de calme. On peut dire comment on souffle. Le cercle irisé tremble encore. La chemise bleue attend sur la corde.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une barre de soleil rampe sur le plancher. Dans la barre, un peu de poussière flotte. Les crayons sentent le bois, près du mur. Une chaise racle, puis s'arrête. Le carton de cartes attend sous la lumière. Dedans, les cartes glissent un peu. Sur le bois de la chaise, un &lt;emphasis level="moderate"&gt;éclat de bois&lt;/emphasis&gt; brille. Il est petit, papa. C'est le bois, sous le soleil. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le cartable attend près de la porte. La fermeture du cartable est un peu froide. Je veux la carte de l'oiseau, maintenant ! Avant de partir ? Oui, tout de suite ! En ce moment, Aniss plonge la main dans le carton. Les cartes glissent contre ses doigts. Une carte tombe, puis une autre. La chaise racle plus fort. Papa parle à maman, près de la porte. Le cartable est près du banc. Oui, avec la fermeture. Papa, l'oiseau ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? La carte va partir. Aniss plonge trop vite, une deuxième fois. Le carton penche, puis se recale. L'oiseau disparaît sous les autres cartes. Oh. L'éclat de bois tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça fait trop de bruit, maman. Ses épaules tombent un peu. Il recule jusqu'au mur. Ses mains touchent le mur, plates. Aniss a besoin de calme. Papa se baisse à sa hauteur. Tu regardes le carton ? Oui, papa. Les crayons sentent le bois, ici. On pioche. On montre. Les deux mots passent trop vite, dans le bruit. Je n'ai pas entendu. Aniss serre le mur contre ses paumes. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Olympe est en classe. Swann explique un jeu de cartes. Olympe reste près du mur. Elle a besoin de calme. Swann va &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. Il dit : on pioche. On montre. Olympe écoute. Elle va observer d'abord. Elle regarde. Elle ne joue pas encore. La maîtresse dit : observer d'abord, c'est possible. Plus tard, Olympe pioche une carte. Maman, le soir, dit : tu as su répéter. Olympe a pu observer d'abord. [pause]</t>
+          <t>Une barre de soleil rampe sur le plancher. Dans la barre, un peu de poussière flotte. Les crayons sentent le bois, près du mur. Une chaise racle, puis s'arrête. Le carton de cartes attend sous la lumière. Dedans, les cartes glissent un peu. Sur le bois de la chaise, un &lt;emphasis&gt;éclat de bois&lt;/emphasis&gt; brille. Il est petit, papa. C'est le bois, sous le soleil. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le cartable attend près de la porte. La fermeture du cartable est un peu froide. Je veux la carte de l'oiseau, maintenant ! Avant de partir ? Oui, tout de suite ! En ce moment, Aniss plonge la main dans le carton. Les cartes glissent contre ses doigts. Une carte tombe, puis une autre. La chaise racle plus fort. Papa parle à maman, près de la porte. Le cartable est près du banc. Oui, avec la fermeture. Papa, l'oiseau ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? La carte va partir. Aniss plonge trop vite, une deuxième fois. Le carton penche, puis se recale. L'oiseau disparaît sous les autres cartes. Oh. L'éclat de bois tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça fait trop de bruit, maman. Ses épaules tombent un peu. Il recule jusqu'au mur. Ses mains touchent le mur, plates. Aniss a besoin de calme. Papa se baisse à sa hauteur. Tu regardes le carton ? Oui, papa. Les crayons sentent le bois, ici. On pioche. On montre. Les deux mots passent trop vite, dans le bruit. Je n'ai pas entendu. Aniss serre le mur contre ses paumes. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de bois</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,43 +1326,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_carte_oiseau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le linge claque sur la corde.
-narrateur|Une goutte tombe d'une chemise bleue.
-narrateur|Le savon sent la fleur, dans le bol.
-narrateur|Un cercle irisé tremble au bord.
-narrateur|La cour est encore chaude.
-maman|Tu as vu la chemise, Aniss ?
-enfant-m|Elle est bleue.
-enfant-m|Une goutte tombe.
-maman|Oui.
-maman|Le linge sèche.
-enfant-m|Je veux une bulle.
-enfant-m|Jusqu'à la chemise.
-maman|On souffle tout doux, alors.
-narrateur|Une pince à linge brille au soleil.
-maman|Tu as vu la pince ?
-enfant-m|Elle est jaune.
-maman|Oui.
-maman|Elle tient la manche.
-narrateur|En ce moment, Aniss rentre de l'école.
-narrateur|La classe était un peu bruyante.
-narrateur|Il reste près du mur.
-narrateur|Le mur est chaud sous sa main.
-narrateur|Raphaël tient déjà l'anneau.
-narrateur|L'anneau goutte un peu de savon.
-enfant-m|J'attends un peu.
-maman|Tu as besoin de calme.
-maman|On peut dire comment on souffle.
-narrateur|Le cercle irisé tremble encore.
-narrateur|La chemise bleue attend sur la corde.</t>
+          <t>narrateur|Une barre de soleil rampe sur le plancher.
+narrateur|Dans la barre, un peu de poussière flotte.
+narrateur|Les crayons sentent le bois, près du mur.
+narrateur|Une chaise racle, puis s'arrête.
+narrateur|Le carton de cartes attend sous la lumière.
+narrateur|Dedans, les cartes glissent un peu.
+narrateur|Sur le bois de la chaise, un éclat de bois brille.
+enfant-m|Il est petit, papa.
+papa|C'est le bois, sous le soleil.
+narrateur|Papa tient la main d'Aniss.
+papa|Ta main est bien dans la mienne.
+maman|Le cartable attend près de la porte.
+narrateur|La fermeture du cartable est un peu froide.
+enfant-m|Je veux la carte de l'oiseau, maintenant !
+maman|Avant de partir ?
+enfant-m|Oui, tout de suite !
+narrateur|En ce moment, Aniss plonge la main dans le carton.
+narrateur|Les cartes glissent contre ses doigts.
+narrateur|Une carte tombe, puis une autre.
+narrateur|La chaise racle plus fort.
+narrateur|Papa parle à maman, près de la porte.
+papa|Le cartable est près du banc.
+maman|Oui, avec la fermeture.
+enfant-m|Papa, l'oiseau !
+narrateur|Les mots d'Aniss se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Aniss ?
+enfant-m|La carte va partir.
+narrateur|Aniss plonge trop vite, une deuxième fois.
+narrateur|Le carton penche, puis se recale.
+narrateur|L'oiseau disparaît sous les autres cartes.
+enfant-m|Oh.
+narrateur|L'éclat de bois tremble, puis tient.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça fait trop de bruit, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Il recule jusqu'au mur.
+narrateur|Ses mains touchent le mur, plates.
+narrateur|Aniss a besoin de calme.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes le carton ?
+enfant-m|Oui, papa.
+maman|Les crayons sentent le bois, ici.
+papa|On pioche.
+papa|On montre.
+narrateur|Les deux mots passent trop vite, dans le bruit.
+enfant-m|Je n'ai pas entendu.
+narrateur|Aniss serre le mur contre ses paumes.
+narrateur|Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>linge,savon</t>
+          <t>chaise,cartes</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Olympe a besoin de calme. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1462,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1473,7 +1498,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1488,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,17 +1559,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_peut_redire_les_mots_plus_lent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>On trempe l'anneau. On souffle tout doux. Maman vient de répéter. Aniss va observer d'abord. Raphaël trempe l'anneau. Il souffle une petite bulle. La bulle part, puis crève. Aniss suit des yeux. Il ne souffle pas encore. Observer d'abord, c'est possible. Plus tard, Aniss tend la main. Il prend l'anneau. Le savon est froid, un peu glissant. Je souffle. Une bulle ronde se détache. Elle va vers la chemise bleue. Elle se pose, une seconde. Elle est arrivée. Bravo, Aniss. Tu as regardé, puis soufflé. Un rond mouillé reste sur le bleu. Puis il s'en va. Elle a touché la manche. Oui. Une seconde, pas plus. Raphaël pose l'anneau au bord du bol. Le savon sent encore la fleur.</t>
+          <t>Papa se rapproche, sans presser. On pioche. On montre. Cette fois, les mots arrivent lents. On pioche. On montre. Aniss regarde le carton, sans y mettre la main. Papa pioche une carte, sans brusquer. Il la montre, près du soleil. C'est un arbre. Je vois l'arbre. Tu as regardé le carton ? Oui, maman. Aniss tend la main, plus légère. Il pioche une carte. C'est l'oiseau. Il la montre, sans la jeter. C'est mon oiseau. Merci, Aniss. Papa a vu l'oiseau, entier. Tu as fini de la montrer ? Oui, maman. Le ventre d'Aniss se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>On trempe l'anneau. On souffle tout doux. Maman vient de répéter. Aniss va observer d'abord. Raphaël trempe l'anneau. Il souffle une petite bulle. La bulle part, puis crève. Aniss suit des yeux. Il ne souffle pas encore. Observer d'abord, c'est possible. Plus tard, Aniss tend la main. Il prend l'anneau. Le savon est froid, un peu glissant. Je souffle. Une bulle ronde se détache. Elle va vers la chemise bleue. Elle se pose, une seconde. Elle est arrivée. Bravo, Aniss. Tu as regardé, puis soufflé. Un rond mouillé reste sur le bleu. Puis il s'en va. Elle a touché la manche. Oui. Une seconde, pas plus. Raphaël pose l'anneau au bord du bol. Le savon sent encore la fleur.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa se rapproche, sans presser. On pioche. On montre. Cette fois, les mots arrivent lents. On pioche. On montre. Aniss regarde le carton, sans y mettre la main. Papa pioche une carte, sans brusquer. Il la montre, près du soleil. C'est un arbre. Je vois l'arbre. Tu as regardé le carton ? Oui, maman. Aniss tend la main, plus légère. Il pioche une carte. C'est l'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;. Il la montre, sans la jeter. C'est mon oiseau. Merci, Aniss. Papa a vu l'oiseau, entier. Tu as fini de la montrer ? Oui, maman. Le ventre d'Aniss se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Swann a répété. Olympe a observé d'abord. Puis elle a joué un peu. [pause]</t>
+          <t>Papa se rapproche, sans presser. On pioche. On montre. Cette fois, les mots arrivent lents. On pioche. On montre. Aniss regarde le carton, sans y mettre la main. Papa pioche une carte, sans brusquer. Il la montre, près du soleil. C'est un arbre. Je vois l'arbre. Tu as regardé le carton ? Oui, maman. Aniss tend la main, plus légère. Il pioche une carte. C'est l'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;. Il la montre, sans la jeter. C'est mon oiseau. Merci, Aniss. Papa a vu l'oiseau, entier. Tu as fini de la montrer ? Oui, maman. Le ventre d'Aniss se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1659,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1667,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1662,28 +1691,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>oiseau</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1692,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1708,43 +1741,39 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=papa_redite_il_observe_puis_pioche; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>maman|On trempe l'anneau.
-maman|On souffle tout doux.
-narrateur|Maman vient de répéter.
-narrateur|Aniss va observer d'abord.
-narrateur|Raphaël trempe l'anneau.
-narrateur|Il souffle une petite bulle.
-narrateur|La bulle part, puis crève.
-narrateur|Aniss suit des yeux.
-narrateur|Il ne souffle pas encore.
-maman|Observer d'abord, c'est possible.
-narrateur|Plus tard, Aniss tend la main.
-narrateur|Il prend l'anneau.
-narrateur|Le savon est froid, un peu glissant.
-enfant-m|Je souffle.
-narrateur|Une bulle ronde se détache.
-narrateur|Elle va vers la chemise bleue.
-narrateur|Elle se pose, une seconde.
-enfant-m|Elle est arrivée.
-maman|Bravo, Aniss.
-maman|Tu as regardé, puis soufflé.
-narrateur|Un rond mouillé reste sur le bleu.
-narrateur|Puis il s'en va.
-enfant-m|Elle a touché la manche.
-maman|Oui.
-maman|Une seconde, pas plus.
-narrateur|Raphaël pose l'anneau au bord du bol.
-narrateur|Le savon sent encore la fleur.</t>
+          <t>narrateur|Papa se rapproche, sans presser.
+papa|On pioche.
+papa|On montre.
+narrateur|Cette fois, les mots arrivent lents.
+enfant-m|On pioche.
+enfant-m|On montre.
+narrateur|Aniss regarde le carton, sans y mettre la main.
+narrateur|Papa pioche une carte, sans brusquer.
+narrateur|Il la montre, près du soleil.
+papa|C'est un arbre.
+enfant-m|Je vois l'arbre.
+maman|Tu as regardé le carton ?
+enfant-m|Oui, maman.
+narrateur|Aniss tend la main, plus légère.
+narrateur|Il pioche une carte.
+narrateur|C'est l'oiseau.
+narrateur|Il la montre, sans la jeter.
+enfant-m|C'est mon oiseau.
+papa|Merci, Aniss.
+narrateur|Papa a vu l'oiseau, entier.
+maman|Tu as fini de la montrer ?
+enfant-m|Oui, maman.
+narrateur|Le ventre d'Aniss se desserre.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>bulle</t>
+          <t>cartes</t>
         </is>
       </c>
     </row>
@@ -1771,17 +1800,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa ouvre le portail. Ça sent le savon, ici. J'ai fait une bulle. Jusqu'à la chemise. Elle est encore là ? Un rond, puis plus rien. Aniss a observé d'abord. Puis il a soufflé. Tu as fini de tenir l'anneau ? Oui, maman. L'anneau rentre dans le bol. Le savon fait un petit ploc. Le linge claque encore. La chemise est presque sèche. On rentre les pinces, maintenant. La cour redevient calme. Le mur n'est plus si chaud. La pince jaune aussi. Oui. Avec les autres. Une goutte tombe encore, puis plus.</t>
+          <t>Aniss veut poser la carte dans le carton. Je la mets, maintenant ! Il envoie la carte trop vite. La carte glisse sous la chaise. Oh. L'oiseau a disparu, sous le bois. Aniss veut ramper tout de suite. Il refuse de foncer. Attends, je regarde. Personne ne parle. Il observe la chaise, puis le plancher. Il écoute le silence de la classe. Sous le pied de la chaise, un éclat de bois brille. Il est là. Comme tout à l'heure. Tu le vois, sur le bois ? Oui, et l'oiseau aussi. Aniss avance la main, plus légère. Il reprend la carte, sans brusquer. L'oiseau est un peu poussiéreux. Il est là, maman. On voit l'oiseau. Et le carton, à côté ? Je le pose, sans jeter. Aniss glisse la carte dans le carton. Les cartes font un petit bruit, puis rien. Ffff. Aniss souffle sur le bois de la chaise.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa ouvre le portail. Ça sent le savon, ici. J'ai fait une bulle. Jusqu'à la chemise. Elle est encore là ? Un rond, puis plus rien. Aniss a observé d'abord. Puis il a soufflé. Tu as fini de tenir l'anneau ? Oui, maman. L'anneau rentre dans le bol. Le savon fait un petit ploc. Le linge claque encore. La chemise est presque sèche. On rentre les pinces, maintenant. La cour redevient calme. Le mur n'est plus si chaud. La pince jaune aussi. Oui. Avec les autres. Une goutte tombe encore, puis plus.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut poser la carte dans le carton. Je la mets, maintenant ! Il envoie la carte trop vite. La carte glisse sous la chaise. Oh. L'oiseau a disparu, sous le bois. Aniss veut ramper tout de suite. Il refuse de foncer. Attends, je regarde. Personne ne parle. Il observe la chaise, puis le plancher. Il écoute le silence de la classe. Sous le pied de la chaise, un &lt;emphasis level="moderate"&gt;éclat de bois&lt;/emphasis&gt; brille. Il est là. Comme tout à l'heure. Tu le vois, sur le bois ? Oui, et l'oiseau aussi. Aniss avance la main, plus légère. Il reprend la carte, sans brusquer. L'oiseau est un peu poussiéreux. Il est là, maman. On voit l'oiseau. Et le carton, à côté ? Je le pose, sans jeter. Aniss glisse la carte dans le carton. Les cartes font un petit bruit, puis rien. Ffff. Aniss souffle sur le bois de la chaise.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range le cartable. Olympe donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Aniss veut poser la carte dans le carton. Je la mets, maintenant ! Il envoie la carte trop vite. La carte glisse sous la chaise. Oh. L'oiseau a disparu, sous le bois. Aniss veut ramper tout de suite. Il refuse de foncer. Attends, je regarde. Personne ne parle. Il observe la chaise, puis le plancher. Il écoute le silence de la classe. Sous le pied de la chaise, un &lt;emphasis&gt;éclat de bois&lt;/emphasis&gt; brille. Il est là. Comme tout à l'heure. Tu le vois, sur le bois ? Oui, et l'oiseau aussi. Aniss avance la main, plus légère. Il reprend la carte, sans brusquer. L'oiseau est un peu poussiéreux. Il est là, maman. On voit l'oiseau. Et le carton, à côté ? Je le pose, sans jeter. Aniss glisse la carte dans le carton. Les cartes font un petit bruit, puis rien. Ffff. Aniss souffle sur le bois de la chaise. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1828,7 +1857,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1836,10 +1865,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1862,30 +1891,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de bois</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1894,10 +1923,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,35 +1937,46 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa ouvre le portail.
-papa|Ça sent le savon, ici.
-enfant-m|J'ai fait une bulle.
-enfant-m|Jusqu'à la chemise.
-papa|Elle est encore là ?
-enfant-m|Un rond, puis plus rien.
-maman|Aniss a observé d'abord.
-papa|Puis il a soufflé.
-maman|Tu as fini de tenir l'anneau ?
-enfant-m|Oui, maman.
-narrateur|L'anneau rentre dans le bol.
-narrateur|Le savon fait un petit ploc.
-papa|Le linge claque encore.
-enfant-m|La chemise est presque sèche.
-maman|On rentre les pinces, maintenant.
-narrateur|La cour redevient calme.
-narrateur|Le mur n'est plus si chaud.
-enfant-m|La pince jaune aussi.
-papa|Oui.
-papa|Avec les autres.
-narrateur|Une goutte tombe encore, puis plus.</t>
+          <t>narrateur|Aniss veut poser la carte dans le carton.
+enfant-m|Je la mets, maintenant !
+narrateur|Il envoie la carte trop vite.
+narrateur|La carte glisse sous la chaise.
+enfant-m|Oh.
+narrateur|L'oiseau a disparu, sous le bois.
+narrateur|Aniss veut ramper tout de suite.
+narrateur|Il refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Personne ne parle.
+narrateur|Il observe la chaise, puis le plancher.
+narrateur|Il écoute le silence de la classe.
+narrateur|Sous le pied de la chaise, un éclat de bois brille.
+enfant-m|Il est là.
+enfant-m|Comme tout à l'heure.
+papa|Tu le vois, sur le bois ?
+enfant-m|Oui, et l'oiseau aussi.
+narrateur|Aniss avance la main, plus légère.
+narrateur|Il reprend la carte, sans brusquer.
+narrateur|L'oiseau est un peu poussiéreux.
+enfant-m|Il est là, maman.
+maman|On voit l'oiseau.
+papa|Et le carton, à côté ?
+enfant-m|Je le pose, sans jeter.
+narrateur|Aniss glisse la carte dans le carton.
+narrateur|Les cartes font un petit bruit, puis rien.
+enfant-m|Ffff.
+narrateur|Aniss souffle sur le bois de la chaise.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>portail,linge</t>
+          <t>chaise,cartes</t>
         </is>
       </c>
     </row>
@@ -1963,17 +2003,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bol repose près du robinet. La chemise bleue sèche encore. Bonne fin de journée, Aniss. La bulle a fait un rond.</t>
+          <t>Le carton repose près de la chaise. L'oiseau reste dedans, avec les autres. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le bois. On est bien, ici. La barre de soleil a bougé, sur le plancher. Aniss glisse la chaise sans se presser. Le bois repose contre le plancher. On le voit, maman. Tu le vois sur le bois ? Oui, l'éclat. Tu as fini de fermer le cartable ? Oui, maman. Le soir reste dans l'air de la classe. L'éclat de bois tient sur la chaise.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bol repose près du robinet. La chemise bleue sèche encore. Bonne fin de journée, Aniss. La bulle a fait un rond.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le carton repose près de la chaise. L'oiseau reste dedans, avec les autres. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le bois. On est bien, ici. La barre de soleil a bougé, sur le plancher. Aniss glisse la chaise sans se presser. Le bois repose contre le plancher. On le voit, maman. Tu le vois sur le bois ? Oui, l'éclat. Tu as fini de fermer le cartable ? Oui, maman. Le soir reste dans l'air de la classe. L'&lt;emphasis level="moderate"&gt;éclat de bois&lt;/emphasis&gt; tient sur la chaise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le carton repose près de la chaise. L'oiseau reste dedans, avec les autres. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le bois. On est bien, ici. La barre de soleil a bougé, sur le plancher. Aniss glisse la chaise sans se presser. Le bois repose contre le plancher. On le voit, maman. Tu le vois sur le bois ? Oui, l'éclat. Tu as fini de fermer le cartable ? Oui, maman. Le soir reste dans l'air de la classe. L'&lt;emphasis&gt;éclat de bois&lt;/emphasis&gt; tient sur la chaise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2020,7 +2060,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2028,10 +2068,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2040,12 +2080,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2054,17 +2094,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bois</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2073,11 +2117,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2086,27 +2130,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_chaise; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bol repose près du robinet.
-narrateur|La chemise bleue sèche encore.
-maman|Bonne fin de journée, Aniss.
-papa|La bulle a fait un rond.</t>
+          <t>narrateur|Le carton repose près de la chaise.
+narrateur|L'oiseau reste dedans, avec les autres.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bois.
+maman|On est bien, ici.
+narrateur|La barre de soleil a bougé, sur le plancher.
+narrateur|Aniss glisse la chaise sans se presser.
+narrateur|Le bois repose contre le plancher.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le bois ?
+enfant-m|Oui, l'éclat.
+maman|Tu as fini de fermer le cartable ?
+enfant-m|Oui, maman.
+narrateur|Le soir reste dans l'air de la classe.
+narrateur|L'éclat de bois tient sur la chaise.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>chaise</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2212,6 +2277,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>